<commit_message>
Siliconomics v0.8：HBM 營收份額表（M24、ShareTbl、K6-hbm）；台積電 HBM 2027 缺口改讀本庫
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V11Bd11jZKXZ5hH5AjB7NJ
</commit_message>
<xml_diff>
--- a/tsmc/dist/20261028_台積電個股模型_v0.4.xlsx
+++ b/tsmc/dist/20261028_台積電個股模型_v0.4.xlsx
@@ -10989,7 +10989,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">markets/memory</t>
+      <t xml:space="preserve">Siliconomics</t>
     </r>
     <r>
       <rPr>
@@ -11010,16 +11010,35 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">markets/memory Mkt</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：需求 </t>
+      <t xml:space="preserve">Siliconomics SIF_HBM_GapEB_A ÷ SIF_HBM_SupplyEB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2027</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）：需求 </t>
     </r>
     <r>
       <rPr>
@@ -39242,7 +39261,7 @@
         <v>42</v>
       </c>
       <c r="E75" s="7" t="n">
-        <v>0.21</v>
+        <v>0.210219254415343</v>
       </c>
       <c r="G75" s="8" t="s">
         <v>128</v>
@@ -42095,7 +42114,7 @@
       </c>
       <c r="C18" s="17" t="n">
         <f aca="false">hbm_gap27</f>
-        <v>0.21</v>
+        <v>0.210219254415343</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>554</v>

</xml_diff>